<commit_message>
Set ad report period to 10/3-10/8
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qcxxm45opVsMXpkD7SANqh
</commit_message>
<xml_diff>
--- a/중국라벨_판매현황_광고테스트.xlsx
+++ b/중국라벨_판매현황_광고테스트.xlsx
@@ -5808,7 +5808,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· </t>
+      <t xml:space="preserve">· 10/3~10/8, 6</t>
     </r>
     <r>
       <rPr>
@@ -5818,7 +5818,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">네이버 검색광고 리포트 </t>
+      <t xml:space="preserve">일 </t>
     </r>
     <r>
       <rPr>
@@ -5829,7 +5829,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">10/8 16:57 </t>
+      <t xml:space="preserve">· </t>
     </r>
     <r>
       <rPr>
@@ -5839,7 +5839,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">다운로드</t>
+      <t xml:space="preserve">네이버 검색광고 리포트</t>
     </r>
     <r>
       <rPr>
@@ -6985,7 +6985,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">. </t>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
@@ -6994,7 +6994,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">조회 기간은 리포트 파일에 표시되지 않습니다</t>
+      <t xml:space="preserve">조회 기간 </t>
     </r>
     <r>
       <rPr>
@@ -7004,7 +7004,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">. </t>
+      <t xml:space="preserve">10/3~10/8). </t>
     </r>
     <r>
       <rPr>
@@ -17948,7 +17948,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N98"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -18495,95 +18495,61 @@
         <v>277</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
+    <row r="23" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H24" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J24" s="3" t="s">
         <v>286</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>287</v>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="G24" s="60" t="n">
-        <f aca="false">E24-C24</f>
-        <v>3</v>
-      </c>
-      <c r="H24" s="60" t="n">
-        <f aca="false">F24-D24</f>
-        <v>10</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="7" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G25" s="60" t="n">
         <f aca="false">E25-C25</f>
@@ -18591,21 +18557,21 @@
       </c>
       <c r="H25" s="60" t="n">
         <f aca="false">F25-D25</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C26" s="7" t="n">
         <v>0</v>
@@ -18617,7 +18583,7 @@
         <v>3</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G26" s="60" t="n">
         <f aca="false">E26-C26</f>
@@ -18625,207 +18591,219 @@
       </c>
       <c r="H26" s="60" t="n">
         <f aca="false">F26-D26</f>
+        <v>7</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>289</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="I26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
+      <c r="G27" s="60" t="n">
+        <f aca="false">E27-C27</f>
+        <v>3</v>
+      </c>
+      <c r="H27" s="60" t="n">
+        <f aca="false">F27-D27</f>
+        <v>17</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="9" t="n">
-        <f aca="false">C24+C25+C26</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="9" t="n">
-        <f aca="false">D24+D25+D26</f>
+      <c r="B28" s="15"/>
+      <c r="C28" s="9" t="n">
+        <f aca="false">C25+C26+C27</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <f aca="false">D25+D26+D27</f>
         <v>5</v>
       </c>
-      <c r="E27" s="9" t="n">
-        <f aca="false">E24+E25+E26</f>
+      <c r="E28" s="9" t="n">
+        <f aca="false">E25+E26+E27</f>
         <v>10</v>
       </c>
-      <c r="F27" s="9" t="n">
-        <f aca="false">F24+F25+F26</f>
+      <c r="F28" s="9" t="n">
+        <f aca="false">F25+F26+F27</f>
         <v>39</v>
       </c>
-      <c r="G27" s="61" t="n">
-        <f aca="false">G24+G25+G26</f>
+      <c r="G28" s="61" t="n">
+        <f aca="false">G25+G26+G27</f>
         <v>9</v>
       </c>
-      <c r="H27" s="61" t="n">
-        <f aca="false">H24+H25+H26</f>
+      <c r="H28" s="61" t="n">
+        <f aca="false">H25+H26+H27</f>
         <v>34</v>
       </c>
-      <c r="I27" s="9" t="n">
-        <f aca="false">I24+I25+I26</f>
+      <c r="I28" s="9" t="n">
+        <f aca="false">I25+I26+I27</f>
         <v>4</v>
       </c>
-      <c r="J27" s="9" t="n">
-        <f aca="false">J24+J25+J26</f>
+      <c r="J28" s="9" t="n">
+        <f aca="false">J25+J26+J27</f>
         <v>8</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="62" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="62" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
+    <row r="32" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="25" t="s">
         <v>293</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-    </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B34" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C34" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3" t="s">
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="63" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B34" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="65" t="s">
+      <c r="B35" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D35" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E34" s="66" t="s">
+      <c r="E35" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F34" s="67" t="s">
+      <c r="F35" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
-      <c r="J34" s="20"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="20"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A36" s="11" t="s">
         <v>302</v>
       </c>
-      <c r="B35" s="35" t="s">
+      <c r="B36" s="35" t="s">
         <v>303</v>
       </c>
-      <c r="C35" s="68" t="s">
+      <c r="C36" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D35" s="68" t="s">
+      <c r="D36" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="69"/>
-      <c r="H35" s="69"/>
-      <c r="I35" s="69"/>
-      <c r="J35" s="69"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="63" t="n">
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
+      <c r="J36" s="69"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="63" t="n">
         <v>2300</v>
       </c>
-      <c r="B36" s="64" t="n">
+      <c r="B37" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="20" t="s">
+      <c r="C37" s="20" t="s">
         <v>305</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="D37" s="20" t="s">
         <v>306</v>
       </c>
-      <c r="E36" s="70" t="s">
+      <c r="E37" s="70" t="s">
         <v>307</v>
       </c>
-      <c r="F36" s="67" t="s">
+      <c r="F37" s="67" t="s">
         <v>308</v>
       </c>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>309</v>
-      </c>
-      <c r="B37" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C37" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D37" s="68" t="s">
-        <v>311</v>
-      </c>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="71" t="s">
-        <v>312</v>
-      </c>
-      <c r="H37" s="71"/>
-      <c r="I37" s="71"/>
-      <c r="J37" s="71"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C38" s="68" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="D38" s="68" t="s">
         <v>311</v>
@@ -18833,160 +18811,162 @@
       <c r="E38" s="22"/>
       <c r="F38" s="22"/>
       <c r="G38" s="71" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="H38" s="71"/>
       <c r="I38" s="71"/>
       <c r="J38" s="71"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="63" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A39" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="C39" s="68" t="s">
+        <v>314</v>
+      </c>
+      <c r="D39" s="68" t="s">
+        <v>311</v>
+      </c>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="71" t="s">
+        <v>315</v>
+      </c>
+      <c r="H39" s="71"/>
+      <c r="I39" s="71"/>
+      <c r="J39" s="71"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="63" t="n">
         <v>2600</v>
       </c>
-      <c r="B39" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="20" t="s">
+      <c r="B40" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D40" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E39" s="66" t="s">
+      <c r="E40" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F39" s="67" t="s">
+      <c r="F40" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A40" s="11" t="s">
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A41" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="B40" s="35" t="s">
+      <c r="B41" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C40" s="68" t="s">
+      <c r="C41" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D40" s="68" t="s">
+      <c r="D41" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="71" t="s">
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="71" t="s">
         <v>319</v>
       </c>
-      <c r="H40" s="71"/>
-      <c r="I40" s="71"/>
-      <c r="J40" s="71"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="63" t="n">
+      <c r="H41" s="71"/>
+      <c r="I41" s="71"/>
+      <c r="J41" s="71"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="63" t="n">
         <v>2800</v>
       </c>
-      <c r="B41" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="20" t="s">
+      <c r="B42" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="D42" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E41" s="70" t="s">
+      <c r="E42" s="70" t="s">
         <v>307</v>
       </c>
-      <c r="F41" s="67" t="s">
+      <c r="F42" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20"/>
-      <c r="I41" s="20"/>
-      <c r="J41" s="20"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A42" s="11" t="s">
+      <c r="G42" s="20"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A43" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="B42" s="35" t="s">
+      <c r="B43" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C42" s="68" t="s">
+      <c r="C43" s="68" t="s">
         <v>314</v>
       </c>
-      <c r="D42" s="68" t="s">
+      <c r="D43" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="71" t="s">
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="71" t="s">
         <v>315</v>
       </c>
-      <c r="H42" s="71"/>
-      <c r="I42" s="71"/>
-      <c r="J42" s="71"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="63" t="n">
+      <c r="H43" s="71"/>
+      <c r="I43" s="71"/>
+      <c r="J43" s="71"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="63" t="n">
         <v>3000</v>
       </c>
-      <c r="B43" s="64" t="n">
+      <c r="B44" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="C44" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D44" s="20" t="s">
         <v>321</v>
       </c>
-      <c r="E43" s="70" t="s">
+      <c r="E44" s="70" t="s">
         <v>307</v>
       </c>
-      <c r="F43" s="67" t="s">
+      <c r="F44" s="67" t="s">
         <v>232</v>
       </c>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="20"/>
-      <c r="J43" s="20"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>322</v>
-      </c>
-      <c r="B44" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C44" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D44" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="69"/>
-      <c r="H44" s="69"/>
-      <c r="I44" s="69"/>
-      <c r="J44" s="69"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="20"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B45" s="35" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C45" s="68" t="s">
         <v>301</v>
       </c>
       <c r="D45" s="68" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="E45" s="22"/>
       <c r="F45" s="22"/>
@@ -18997,16 +18977,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B46" s="35" t="s">
         <v>310</v>
       </c>
       <c r="C46" s="68" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="D46" s="68" t="s">
-        <v>304</v>
+        <v>324</v>
       </c>
       <c r="E46" s="22"/>
       <c r="F46" s="22"/>
@@ -19015,275 +18995,273 @@
       <c r="I46" s="69"/>
       <c r="J46" s="69"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="25" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="C47" s="68" t="s">
+        <v>314</v>
+      </c>
+      <c r="D47" s="68" t="s">
+        <v>304</v>
+      </c>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="69"/>
+      <c r="J47" s="69"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="25" t="s">
         <v>326</v>
       </c>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="28"/>
-      <c r="H48" s="28"/>
-      <c r="I48" s="28"/>
-      <c r="J48" s="28"/>
-    </row>
-    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="28"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="28"/>
+      <c r="I49" s="28"/>
+      <c r="J49" s="28"/>
+    </row>
+    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B50" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C50" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D50" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E50" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="F50" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3" t="s">
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="63" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="63" t="n">
         <v>1500</v>
       </c>
-      <c r="B50" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" s="65" t="s">
+      <c r="B51" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D50" s="20" t="s">
+      <c r="D51" s="20" t="s">
         <v>327</v>
       </c>
-      <c r="E50" s="66" t="s">
+      <c r="E51" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F50" s="67" t="s">
+      <c r="F51" s="67" t="s">
         <v>301</v>
       </c>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="20"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A51" s="11" t="s">
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A52" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="B51" s="35" t="s">
+      <c r="B52" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C51" s="68" t="s">
+      <c r="C52" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D51" s="68" t="s">
+      <c r="D52" s="68" t="s">
         <v>329</v>
       </c>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="71" t="s">
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="71" t="s">
         <v>330</v>
       </c>
-      <c r="H51" s="71"/>
-      <c r="I51" s="71"/>
-      <c r="J51" s="71"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="63" t="n">
+      <c r="H52" s="71"/>
+      <c r="I52" s="71"/>
+      <c r="J52" s="71"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B52" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" s="65" t="s">
+      <c r="B53" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D52" s="20" t="s">
+      <c r="D53" s="20" t="s">
         <v>327</v>
       </c>
-      <c r="E52" s="66" t="s">
+      <c r="E53" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F52" s="67" t="s">
+      <c r="F53" s="67" t="s">
         <v>301</v>
       </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A53" s="11" t="s">
+      <c r="G53" s="20"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A54" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="B53" s="35" t="s">
+      <c r="B54" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C53" s="68" t="s">
+      <c r="C54" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D53" s="68" t="s">
+      <c r="D54" s="68" t="s">
         <v>329</v>
       </c>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="69"/>
-      <c r="H53" s="69"/>
-      <c r="I53" s="69"/>
-      <c r="J53" s="69"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="63" t="n">
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="69"/>
+      <c r="H54" s="69"/>
+      <c r="I54" s="69"/>
+      <c r="J54" s="69"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="63" t="n">
         <v>2500</v>
       </c>
-      <c r="B54" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" s="65" t="s">
+      <c r="B55" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D54" s="20" t="s">
+      <c r="D55" s="20" t="s">
         <v>327</v>
       </c>
-      <c r="E54" s="66" t="s">
+      <c r="E55" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F54" s="67" t="s">
+      <c r="F55" s="67" t="s">
         <v>301</v>
       </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20"/>
-      <c r="J54" s="20"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A55" s="11" t="s">
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="20"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A56" s="11" t="s">
         <v>332</v>
       </c>
-      <c r="B55" s="35" t="s">
+      <c r="B56" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C55" s="68" t="s">
+      <c r="C56" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D55" s="68" t="s">
+      <c r="D56" s="68" t="s">
         <v>329</v>
       </c>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="69"/>
-      <c r="H55" s="69"/>
-      <c r="I55" s="69"/>
-      <c r="J55" s="69"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="63" t="n">
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="69"/>
+      <c r="H56" s="69"/>
+      <c r="I56" s="69"/>
+      <c r="J56" s="69"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="63" t="n">
         <v>2800</v>
       </c>
-      <c r="B56" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="20" t="s">
+      <c r="B57" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D56" s="20" t="s">
+      <c r="D57" s="20" t="s">
         <v>308</v>
       </c>
-      <c r="E56" s="66" t="s">
+      <c r="E57" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F56" s="67" t="s">
+      <c r="F57" s="67" t="s">
         <v>308</v>
       </c>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A57" s="11" t="s">
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A58" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="B57" s="35" t="s">
+      <c r="B58" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C57" s="68" t="s">
+      <c r="C58" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D57" s="68" t="s">
+      <c r="D58" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="71" t="s">
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="71" t="s">
         <v>334</v>
       </c>
-      <c r="H57" s="71"/>
-      <c r="I57" s="71"/>
-      <c r="J57" s="71"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="63" t="n">
+      <c r="H58" s="71"/>
+      <c r="I58" s="71"/>
+      <c r="J58" s="71"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="63" t="n">
         <v>3000</v>
       </c>
-      <c r="B58" s="64" t="n">
+      <c r="B59" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C58" s="65" t="s">
+      <c r="C59" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D58" s="20" t="s">
+      <c r="D59" s="20" t="s">
         <v>335</v>
       </c>
-      <c r="E58" s="66" t="s">
+      <c r="E59" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F58" s="67" t="s">
+      <c r="F59" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="20"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A59" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="B59" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C59" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D59" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="71" t="s">
-        <v>337</v>
-      </c>
-      <c r="H59" s="71"/>
-      <c r="I59" s="71"/>
-      <c r="J59" s="71"/>
+      <c r="G59" s="20"/>
+      <c r="H59" s="20"/>
+      <c r="I59" s="20"/>
+      <c r="J59" s="20"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="B60" s="35" t="s">
         <v>310</v>
@@ -19292,111 +19270,113 @@
         <v>301</v>
       </c>
       <c r="D60" s="68" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="E60" s="22"/>
       <c r="F60" s="22"/>
-      <c r="G60" s="69"/>
-      <c r="H60" s="69"/>
-      <c r="I60" s="69"/>
-      <c r="J60" s="69"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="63" t="n">
+      <c r="G60" s="71" t="s">
+        <v>337</v>
+      </c>
+      <c r="H60" s="71"/>
+      <c r="I60" s="71"/>
+      <c r="J60" s="71"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A61" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="B61" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="C61" s="68" t="s">
+        <v>301</v>
+      </c>
+      <c r="D61" s="68" t="s">
+        <v>311</v>
+      </c>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="69"/>
+      <c r="H61" s="69"/>
+      <c r="I61" s="69"/>
+      <c r="J61" s="69"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="63" t="n">
         <v>3100</v>
       </c>
-      <c r="B61" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C61" s="20" t="s">
+      <c r="B62" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D61" s="20" t="s">
+      <c r="D62" s="20" t="s">
         <v>308</v>
       </c>
-      <c r="E61" s="66" t="s">
+      <c r="E62" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F61" s="67" t="s">
+      <c r="F62" s="67" t="s">
         <v>308</v>
       </c>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A62" s="11" t="s">
+      <c r="G62" s="20"/>
+      <c r="H62" s="20"/>
+      <c r="I62" s="20"/>
+      <c r="J62" s="20"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A63" s="11" t="s">
         <v>338</v>
       </c>
-      <c r="B62" s="35" t="s">
+      <c r="B63" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C62" s="68" t="s">
+      <c r="C63" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D62" s="68" t="s">
+      <c r="D63" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="71" t="s">
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="71" t="s">
         <v>339</v>
       </c>
-      <c r="H62" s="71"/>
-      <c r="I62" s="71"/>
-      <c r="J62" s="71"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="63" t="n">
+      <c r="H63" s="71"/>
+      <c r="I63" s="71"/>
+      <c r="J63" s="71"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="63" t="n">
         <v>3500</v>
       </c>
-      <c r="B63" s="64" t="n">
+      <c r="B64" s="64" t="n">
         <v>4</v>
       </c>
-      <c r="C63" s="20" t="s">
+      <c r="C64" s="20" t="s">
         <v>340</v>
       </c>
-      <c r="D63" s="20" t="s">
+      <c r="D64" s="20" t="s">
         <v>341</v>
       </c>
-      <c r="E63" s="70" t="s">
+      <c r="E64" s="70" t="s">
         <v>307</v>
       </c>
-      <c r="F63" s="67" t="s">
+      <c r="F64" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G63" s="20"/>
-      <c r="H63" s="20"/>
-      <c r="I63" s="20"/>
-      <c r="J63" s="20"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A64" s="11" t="s">
-        <v>342</v>
-      </c>
-      <c r="B64" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C64" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D64" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="69"/>
-      <c r="H64" s="69"/>
-      <c r="I64" s="69"/>
-      <c r="J64" s="69"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="20"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B65" s="35" t="s">
-        <v>344</v>
+        <v>310</v>
       </c>
       <c r="C65" s="68" t="s">
         <v>301</v>
@@ -19413,183 +19393,183 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>310</v>
+        <v>344</v>
       </c>
       <c r="C66" s="68" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
       <c r="D66" s="68" t="s">
         <v>304</v>
       </c>
       <c r="E66" s="22"/>
       <c r="F66" s="22"/>
-      <c r="G66" s="71" t="s">
-        <v>339</v>
-      </c>
-      <c r="H66" s="71"/>
-      <c r="I66" s="71"/>
-      <c r="J66" s="71"/>
+      <c r="G66" s="69"/>
+      <c r="H66" s="69"/>
+      <c r="I66" s="69"/>
+      <c r="J66" s="69"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
       <c r="B67" s="35" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C67" s="68" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="D67" s="68" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="E67" s="22"/>
       <c r="F67" s="22"/>
       <c r="G67" s="71" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="H67" s="71"/>
       <c r="I67" s="71"/>
       <c r="J67" s="71"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="63" t="n">
+    <row r="68" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A68" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B68" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="C68" s="68" t="s">
+        <v>314</v>
+      </c>
+      <c r="D68" s="68" t="s">
+        <v>311</v>
+      </c>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="71" t="s">
+        <v>346</v>
+      </c>
+      <c r="H68" s="71"/>
+      <c r="I68" s="71"/>
+      <c r="J68" s="71"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="63" t="n">
         <v>4000</v>
       </c>
-      <c r="B68" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C68" s="20" t="s">
+      <c r="B69" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="D69" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E68" s="70" t="s">
+      <c r="E69" s="70" t="s">
         <v>307</v>
       </c>
-      <c r="F68" s="67" t="s">
+      <c r="F69" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G68" s="20"/>
-      <c r="H68" s="20"/>
-      <c r="I68" s="20"/>
-      <c r="J68" s="20"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A69" s="11" t="s">
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A70" s="11" t="s">
         <v>325</v>
       </c>
-      <c r="B69" s="35" t="s">
+      <c r="B70" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C69" s="68" t="s">
+      <c r="C70" s="68" t="s">
         <v>314</v>
       </c>
-      <c r="D69" s="68" t="s">
+      <c r="D70" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="69"/>
-      <c r="H69" s="69"/>
-      <c r="I69" s="69"/>
-      <c r="J69" s="69"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="63" t="n">
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="69"/>
+      <c r="H70" s="69"/>
+      <c r="I70" s="69"/>
+      <c r="J70" s="69"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="63" t="n">
         <v>5000</v>
       </c>
-      <c r="B70" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C70" s="65" t="s">
+      <c r="B71" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D70" s="20" t="s">
+      <c r="D71" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E70" s="66" t="s">
+      <c r="E71" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F70" s="67" t="s">
+      <c r="F71" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G70" s="20"/>
-      <c r="H70" s="20"/>
-      <c r="I70" s="20"/>
-      <c r="J70" s="20"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A71" s="11" t="s">
+      <c r="G71" s="20"/>
+      <c r="H71" s="20"/>
+      <c r="I71" s="20"/>
+      <c r="J71" s="20"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A72" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="B71" s="35" t="s">
+      <c r="B72" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C71" s="68" t="s">
+      <c r="C72" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D71" s="68" t="s">
+      <c r="D72" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
-      <c r="G71" s="69"/>
-      <c r="H71" s="69"/>
-      <c r="I71" s="69"/>
-      <c r="J71" s="69"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="63" t="n">
+      <c r="E72" s="22"/>
+      <c r="F72" s="22"/>
+      <c r="G72" s="69"/>
+      <c r="H72" s="69"/>
+      <c r="I72" s="69"/>
+      <c r="J72" s="69"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="63" t="n">
         <v>5500</v>
       </c>
-      <c r="B72" s="64" t="n">
+      <c r="B73" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C72" s="65" t="s">
+      <c r="C73" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D72" s="20" t="s">
+      <c r="D73" s="20" t="s">
         <v>347</v>
       </c>
-      <c r="E72" s="66" t="s">
+      <c r="E73" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F72" s="67" t="s">
+      <c r="F73" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G72" s="20"/>
-      <c r="H72" s="20"/>
-      <c r="I72" s="20"/>
-      <c r="J72" s="20"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A73" s="11" t="s">
-        <v>348</v>
-      </c>
-      <c r="B73" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C73" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D73" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E73" s="22"/>
-      <c r="F73" s="22"/>
-      <c r="G73" s="69"/>
-      <c r="H73" s="69"/>
-      <c r="I73" s="69"/>
-      <c r="J73" s="69"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="20"/>
+      <c r="I73" s="20"/>
+      <c r="J73" s="20"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A74" s="11" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B74" s="35" t="s">
         <v>310</v>
@@ -19607,137 +19587,137 @@
       <c r="I74" s="69"/>
       <c r="J74" s="69"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="63" t="n">
+    <row r="75" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A75" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="B75" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="C75" s="68" t="s">
+        <v>301</v>
+      </c>
+      <c r="D75" s="68" t="s">
+        <v>304</v>
+      </c>
+      <c r="E75" s="22"/>
+      <c r="F75" s="22"/>
+      <c r="G75" s="69"/>
+      <c r="H75" s="69"/>
+      <c r="I75" s="69"/>
+      <c r="J75" s="69"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="63" t="n">
         <v>6000</v>
       </c>
-      <c r="B75" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C75" s="65" t="s">
+      <c r="B76" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D75" s="20" t="s">
+      <c r="D76" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E75" s="66" t="s">
+      <c r="E76" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F75" s="67" t="s">
+      <c r="F76" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G75" s="20"/>
-      <c r="H75" s="20"/>
-      <c r="I75" s="20"/>
-      <c r="J75" s="20"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A76" s="11" t="s">
+      <c r="G76" s="20"/>
+      <c r="H76" s="20"/>
+      <c r="I76" s="20"/>
+      <c r="J76" s="20"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A77" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="B76" s="35" t="s">
+      <c r="B77" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C76" s="68" t="s">
+      <c r="C77" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="D76" s="68" t="s">
+      <c r="D77" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E76" s="22"/>
-      <c r="F76" s="22"/>
-      <c r="G76" s="69"/>
-      <c r="H76" s="69"/>
-      <c r="I76" s="69"/>
-      <c r="J76" s="69"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="25" t="s">
+      <c r="E77" s="22"/>
+      <c r="F77" s="22"/>
+      <c r="G77" s="69"/>
+      <c r="H77" s="69"/>
+      <c r="I77" s="69"/>
+      <c r="J77" s="69"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="25" t="s">
         <v>351</v>
       </c>
-      <c r="B78" s="28"/>
-      <c r="C78" s="28"/>
-      <c r="D78" s="28"/>
-      <c r="E78" s="28"/>
-      <c r="F78" s="28"/>
-      <c r="G78" s="28"/>
-      <c r="H78" s="28"/>
-      <c r="I78" s="28"/>
-      <c r="J78" s="28"/>
-    </row>
-    <row r="79" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
+      <c r="B79" s="28"/>
+      <c r="C79" s="28"/>
+      <c r="D79" s="28"/>
+      <c r="E79" s="28"/>
+      <c r="F79" s="28"/>
+      <c r="G79" s="28"/>
+      <c r="H79" s="28"/>
+      <c r="I79" s="28"/>
+      <c r="J79" s="28"/>
+    </row>
+    <row r="80" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B80" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C80" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D79" s="3" t="s">
+      <c r="D80" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E79" s="3" t="s">
+      <c r="E80" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="F80" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G79" s="3"/>
-      <c r="H79" s="3"/>
-      <c r="I79" s="3"/>
-      <c r="J79" s="3" t="s">
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="63" t="n">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B80" s="64" t="n">
+      <c r="B81" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C80" s="65" t="s">
+      <c r="C81" s="65" t="s">
         <v>300</v>
       </c>
-      <c r="D80" s="20" t="s">
+      <c r="D81" s="20" t="s">
         <v>352</v>
       </c>
-      <c r="E80" s="66" t="s">
+      <c r="E81" s="66" t="s">
         <v>301</v>
       </c>
-      <c r="F80" s="67" t="s">
+      <c r="F81" s="67" t="s">
         <v>301</v>
       </c>
-      <c r="G80" s="20"/>
-      <c r="H80" s="20"/>
-      <c r="I80" s="20"/>
-      <c r="J80" s="20"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A81" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="B81" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C81" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D81" s="68" t="s">
-        <v>329</v>
-      </c>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
-      <c r="G81" s="69"/>
-      <c r="H81" s="69"/>
-      <c r="I81" s="69"/>
-      <c r="J81" s="69"/>
+      <c r="G81" s="20"/>
+      <c r="H81" s="20"/>
+      <c r="I81" s="20"/>
+      <c r="J81" s="20"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A82" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B82" s="35" t="s">
         <v>310</v>
@@ -19755,194 +19735,192 @@
       <c r="I82" s="69"/>
       <c r="J82" s="69"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="63" t="n">
+    <row r="83" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A83" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B83" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="C83" s="68" t="s">
+        <v>301</v>
+      </c>
+      <c r="D83" s="68" t="s">
+        <v>329</v>
+      </c>
+      <c r="E83" s="22"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="69"/>
+      <c r="H83" s="69"/>
+      <c r="I83" s="69"/>
+      <c r="J83" s="69"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="63" t="n">
         <v>2500</v>
       </c>
-      <c r="B83" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C83" s="20" t="s">
+      <c r="B84" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D83" s="20" t="s">
+      <c r="D84" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="E83" s="66" t="s">
+      <c r="E84" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F83" s="67" t="s">
+      <c r="F84" s="67" t="s">
         <v>232</v>
       </c>
-      <c r="G83" s="20"/>
-      <c r="H83" s="20"/>
-      <c r="I83" s="20"/>
-      <c r="J83" s="20"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A84" s="11" t="s">
+      <c r="G84" s="20"/>
+      <c r="H84" s="20"/>
+      <c r="I84" s="20"/>
+      <c r="J84" s="20"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A85" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="B84" s="35" t="s">
+      <c r="B85" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C84" s="68" t="s">
+      <c r="C85" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D84" s="68" t="s">
+      <c r="D85" s="68" t="s">
         <v>314</v>
       </c>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="69"/>
-      <c r="H84" s="69"/>
-      <c r="I84" s="69"/>
-      <c r="J84" s="69"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="63" t="n">
+      <c r="E85" s="22"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="69"/>
+      <c r="H85" s="69"/>
+      <c r="I85" s="69"/>
+      <c r="J85" s="69"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="63" t="n">
         <v>2800</v>
       </c>
-      <c r="B85" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C85" s="20" t="s">
+      <c r="B86" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D85" s="20" t="s">
+      <c r="D86" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="E85" s="66" t="s">
+      <c r="E86" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F85" s="67" t="s">
+      <c r="F86" s="67" t="s">
         <v>354</v>
       </c>
-      <c r="G85" s="20"/>
-      <c r="H85" s="20"/>
-      <c r="I85" s="20"/>
-      <c r="J85" s="20"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A86" s="11" t="s">
+      <c r="G86" s="20"/>
+      <c r="H86" s="20"/>
+      <c r="I86" s="20"/>
+      <c r="J86" s="20"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A87" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="B86" s="35" t="s">
+      <c r="B87" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C86" s="68" t="s">
+      <c r="C87" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D86" s="68" t="s">
+      <c r="D87" s="68" t="s">
         <v>356</v>
       </c>
-      <c r="E86" s="22"/>
-      <c r="F86" s="22"/>
-      <c r="G86" s="71" t="s">
+      <c r="E87" s="22"/>
+      <c r="F87" s="22"/>
+      <c r="G87" s="71" t="s">
         <v>357</v>
       </c>
-      <c r="H86" s="71"/>
-      <c r="I86" s="71"/>
-      <c r="J86" s="71"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="63" t="n">
+      <c r="H87" s="71"/>
+      <c r="I87" s="71"/>
+      <c r="J87" s="71"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="63" t="n">
         <v>3100</v>
       </c>
-      <c r="B87" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C87" s="20" t="s">
+      <c r="B88" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" s="20" t="s">
         <v>358</v>
       </c>
-      <c r="D87" s="20" t="s">
+      <c r="D88" s="20" t="s">
         <v>308</v>
       </c>
-      <c r="E87" s="66" t="s">
+      <c r="E88" s="66" t="s">
         <v>359</v>
       </c>
-      <c r="F87" s="67" t="s">
+      <c r="F88" s="67" t="s">
         <v>308</v>
       </c>
-      <c r="G87" s="20"/>
-      <c r="H87" s="20"/>
-      <c r="I87" s="20"/>
-      <c r="J87" s="20"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A88" s="11" t="s">
+      <c r="G88" s="20"/>
+      <c r="H88" s="20"/>
+      <c r="I88" s="20"/>
+      <c r="J88" s="20"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A89" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="B88" s="35" t="s">
+      <c r="B89" s="35" t="s">
         <v>318</v>
       </c>
-      <c r="C88" s="68" t="s">
+      <c r="C89" s="68" t="s">
         <v>324</v>
       </c>
-      <c r="D88" s="68" t="s">
+      <c r="D89" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
-      <c r="G88" s="71" t="s">
+      <c r="E89" s="22"/>
+      <c r="F89" s="22"/>
+      <c r="G89" s="71" t="s">
         <v>361</v>
       </c>
-      <c r="H88" s="71"/>
-      <c r="I88" s="71"/>
-      <c r="J88" s="71"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="63" t="n">
+      <c r="H89" s="71"/>
+      <c r="I89" s="71"/>
+      <c r="J89" s="71"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="63" t="n">
         <v>3500</v>
       </c>
-      <c r="B89" s="64" t="n">
+      <c r="B90" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C89" s="20" t="s">
+      <c r="C90" s="20" t="s">
         <v>347</v>
       </c>
-      <c r="D89" s="20" t="s">
+      <c r="D90" s="20" t="s">
         <v>347</v>
       </c>
-      <c r="E89" s="66" t="s">
+      <c r="E90" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F89" s="67" t="s">
+      <c r="F90" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G89" s="20"/>
-      <c r="H89" s="20"/>
-      <c r="I89" s="20"/>
-      <c r="J89" s="20"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A90" s="11" t="s">
-        <v>345</v>
-      </c>
-      <c r="B90" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C90" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D90" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E90" s="22"/>
-      <c r="F90" s="22"/>
-      <c r="G90" s="71" t="s">
-        <v>362</v>
-      </c>
-      <c r="H90" s="71"/>
-      <c r="I90" s="71"/>
-      <c r="J90" s="71"/>
+      <c r="G90" s="20"/>
+      <c r="H90" s="20"/>
+      <c r="I90" s="20"/>
+      <c r="J90" s="20"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
       <c r="B91" s="35" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C91" s="68" t="s">
         <v>304</v>
@@ -19953,144 +19931,166 @@
       <c r="E91" s="22"/>
       <c r="F91" s="22"/>
       <c r="G91" s="71" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H91" s="71"/>
       <c r="I91" s="71"/>
       <c r="J91" s="71"/>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="63" t="n">
+    <row r="92" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A92" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B92" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="C92" s="68" t="s">
+        <v>304</v>
+      </c>
+      <c r="D92" s="68" t="s">
+        <v>304</v>
+      </c>
+      <c r="E92" s="22"/>
+      <c r="F92" s="22"/>
+      <c r="G92" s="71" t="s">
+        <v>363</v>
+      </c>
+      <c r="H92" s="71"/>
+      <c r="I92" s="71"/>
+      <c r="J92" s="71"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="63" t="n">
         <v>3700</v>
       </c>
-      <c r="B92" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C92" s="20" t="s">
+      <c r="B93" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="20" t="s">
         <v>358</v>
       </c>
-      <c r="D92" s="20" t="s">
+      <c r="D93" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E92" s="66" t="s">
+      <c r="E93" s="66" t="s">
         <v>359</v>
       </c>
-      <c r="F92" s="67" t="s">
+      <c r="F93" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G92" s="20"/>
-      <c r="H92" s="20"/>
-      <c r="I92" s="20"/>
-      <c r="J92" s="20"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A93" s="11" t="s">
+      <c r="G93" s="20"/>
+      <c r="H93" s="20"/>
+      <c r="I93" s="20"/>
+      <c r="J93" s="20"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A94" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="B93" s="35" t="s">
+      <c r="B94" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C93" s="68" t="s">
+      <c r="C94" s="68" t="s">
         <v>324</v>
       </c>
-      <c r="D93" s="68" t="s">
+      <c r="D94" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E93" s="22"/>
-      <c r="F93" s="22"/>
-      <c r="G93" s="71" t="s">
+      <c r="E94" s="22"/>
+      <c r="F94" s="22"/>
+      <c r="G94" s="71" t="s">
         <v>361</v>
       </c>
-      <c r="H93" s="71"/>
-      <c r="I93" s="71"/>
-      <c r="J93" s="71"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="63" t="n">
+      <c r="H94" s="71"/>
+      <c r="I94" s="71"/>
+      <c r="J94" s="71"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="63" t="n">
         <v>3900</v>
       </c>
-      <c r="B94" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C94" s="20" t="s">
+      <c r="B95" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D94" s="20" t="s">
+      <c r="D95" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E94" s="66" t="s">
+      <c r="E95" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="F94" s="67" t="s">
+      <c r="F95" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G94" s="20"/>
-      <c r="H94" s="20"/>
-      <c r="I94" s="20"/>
-      <c r="J94" s="20"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A95" s="11" t="s">
+      <c r="G95" s="20"/>
+      <c r="H95" s="20"/>
+      <c r="I95" s="20"/>
+      <c r="J95" s="20"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A96" s="11" t="s">
         <v>365</v>
       </c>
-      <c r="B95" s="35" t="s">
+      <c r="B96" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="C95" s="68" t="s">
+      <c r="C96" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D95" s="68" t="s">
+      <c r="D96" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="E95" s="22"/>
-      <c r="F95" s="22"/>
-      <c r="G95" s="71" t="s">
+      <c r="E96" s="22"/>
+      <c r="F96" s="22"/>
+      <c r="G96" s="71" t="s">
         <v>363</v>
       </c>
-      <c r="H95" s="71"/>
-      <c r="I95" s="71"/>
-      <c r="J95" s="71"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2" t="s">
+      <c r="H96" s="71"/>
+      <c r="I96" s="71"/>
+      <c r="J96" s="71"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="s">
         <v>366</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="G36:J36"/>
     <mergeCell ref="G38:J38"/>
-    <mergeCell ref="G40:J40"/>
-    <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="G43:J43"/>
     <mergeCell ref="G45:J45"/>
     <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G53:J53"/>
-    <mergeCell ref="G55:J55"/>
-    <mergeCell ref="G57:J57"/>
-    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G52:J52"/>
+    <mergeCell ref="G54:J54"/>
+    <mergeCell ref="G56:J56"/>
+    <mergeCell ref="G58:J58"/>
     <mergeCell ref="G60:J60"/>
-    <mergeCell ref="G62:J62"/>
-    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="G63:J63"/>
     <mergeCell ref="G65:J65"/>
     <mergeCell ref="G66:J66"/>
     <mergeCell ref="G67:J67"/>
-    <mergeCell ref="G69:J69"/>
-    <mergeCell ref="G71:J71"/>
-    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G68:J68"/>
+    <mergeCell ref="G70:J70"/>
+    <mergeCell ref="G72:J72"/>
     <mergeCell ref="G74:J74"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="G81:J81"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="G77:J77"/>
     <mergeCell ref="G82:J82"/>
-    <mergeCell ref="G84:J84"/>
-    <mergeCell ref="G86:J86"/>
-    <mergeCell ref="G88:J88"/>
-    <mergeCell ref="G90:J90"/>
+    <mergeCell ref="G83:J83"/>
+    <mergeCell ref="G85:J85"/>
+    <mergeCell ref="G87:J87"/>
+    <mergeCell ref="G89:J89"/>
     <mergeCell ref="G91:J91"/>
-    <mergeCell ref="G93:J93"/>
-    <mergeCell ref="G95:J95"/>
+    <mergeCell ref="G92:J92"/>
+    <mergeCell ref="G94:J94"/>
+    <mergeCell ref="G96:J96"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Show daily ad cost note in ad sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qcxxm45opVsMXpkD7SANqh
</commit_message>
<xml_diff>
--- a/중국라벨_판매현황_광고테스트.xlsx
+++ b/중국라벨_판매현황_광고테스트.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="368">
   <si>
     <r>
       <rPr>
@@ -7062,6 +7062,150 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">하루 평균 광고비</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">라벨 광고 상품 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) = 217,167</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">÷ 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일 ≈ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">36,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일이면 약 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">109</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF5A6270"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">만 원</t>
     </r>
   </si>
   <si>
@@ -17948,7 +18092,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N98"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -18495,61 +18639,100 @@
         <v>277</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+    <row r="22" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="D24" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="J24" s="3" t="s">
+      <c r="I23" s="3" t="s">
         <v>286</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" s="60" t="n">
+        <f aca="false">E24-C24</f>
+        <v>3</v>
+      </c>
+      <c r="H24" s="60" t="n">
+        <f aca="false">F24-D24</f>
+        <v>10</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G25" s="60" t="n">
         <f aca="false">E25-C25</f>
@@ -18557,21 +18740,21 @@
       </c>
       <c r="H25" s="60" t="n">
         <f aca="false">F25-D25</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C26" s="7" t="n">
         <v>0</v>
@@ -18583,7 +18766,7 @@
         <v>3</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G26" s="60" t="n">
         <f aca="false">E26-C26</f>
@@ -18591,382 +18774,368 @@
       </c>
       <c r="H26" s="60" t="n">
         <f aca="false">F26-D26</f>
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>289</v>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="G27" s="60" t="n">
-        <f aca="false">E27-C27</f>
-        <v>3</v>
-      </c>
-      <c r="H27" s="60" t="n">
-        <f aca="false">F27-D27</f>
-        <v>17</v>
-      </c>
-      <c r="I27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <v>0</v>
+      <c r="A27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="15"/>
+      <c r="C27" s="9" t="n">
+        <f aca="false">C24+C25+C26</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <f aca="false">D24+D25+D26</f>
+        <v>5</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <f aca="false">E24+E25+E26</f>
+        <v>10</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <f aca="false">F24+F25+F26</f>
+        <v>39</v>
+      </c>
+      <c r="G27" s="61" t="n">
+        <f aca="false">G24+G25+G26</f>
+        <v>9</v>
+      </c>
+      <c r="H27" s="61" t="n">
+        <f aca="false">H24+H25+H26</f>
+        <v>34</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <f aca="false">I24+I25+I26</f>
+        <v>4</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <f aca="false">J24+J25+J26</f>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="9" t="n">
-        <f aca="false">C25+C26+C27</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <f aca="false">D25+D26+D27</f>
-        <v>5</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <f aca="false">E25+E26+E27</f>
-        <v>10</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <f aca="false">F25+F26+F27</f>
-        <v>39</v>
-      </c>
-      <c r="G28" s="61" t="n">
-        <f aca="false">G25+G26+G27</f>
-        <v>9</v>
-      </c>
-      <c r="H28" s="61" t="n">
-        <f aca="false">H25+H26+H27</f>
-        <v>34</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <f aca="false">I25+I26+I27</f>
-        <v>4</v>
-      </c>
-      <c r="J28" s="9" t="n">
-        <f aca="false">J25+J26+J27</f>
-        <v>8</v>
+      <c r="A28" s="2" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="62" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
+      <c r="A29" s="62" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
+    <row r="31" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="28"/>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B34" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B33" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="C33" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="63" t="n">
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B35" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D35" s="20" t="s">
+      <c r="B34" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="65" t="s">
+        <v>301</v>
+      </c>
+      <c r="D34" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E35" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F35" s="67" t="s">
+      <c r="E34" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F34" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
-      <c r="J35" s="20"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A36" s="11" t="s">
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="20"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>304</v>
+      </c>
+      <c r="C35" s="68" t="s">
         <v>302</v>
       </c>
-      <c r="B36" s="35" t="s">
-        <v>303</v>
-      </c>
-      <c r="C36" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D36" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="69"/>
-      <c r="I36" s="69"/>
-      <c r="J36" s="69"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="63" t="n">
+      <c r="D35" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="69"/>
+      <c r="H35" s="69"/>
+      <c r="I35" s="69"/>
+      <c r="J35" s="69"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="63" t="n">
         <v>2300</v>
       </c>
-      <c r="B37" s="64" t="n">
+      <c r="B36" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C37" s="20" t="s">
+      <c r="C36" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="E36" s="70" t="s">
+        <v>308</v>
+      </c>
+      <c r="F36" s="67" t="s">
+        <v>309</v>
+      </c>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C37" s="68" t="s">
         <v>305</v>
       </c>
-      <c r="D37" s="20" t="s">
-        <v>306</v>
-      </c>
-      <c r="E37" s="70" t="s">
-        <v>307</v>
-      </c>
-      <c r="F37" s="67" t="s">
-        <v>308</v>
-      </c>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20"/>
+      <c r="D37" s="68" t="s">
+        <v>312</v>
+      </c>
+      <c r="E37" s="22"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="71" t="s">
+        <v>313</v>
+      </c>
+      <c r="H37" s="71"/>
+      <c r="I37" s="71"/>
+      <c r="J37" s="71"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C38" s="68" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="D38" s="68" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E38" s="22"/>
       <c r="F38" s="22"/>
       <c r="G38" s="71" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="H38" s="71"/>
       <c r="I38" s="71"/>
       <c r="J38" s="71"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>313</v>
-      </c>
-      <c r="B39" s="35" t="s">
-        <v>303</v>
-      </c>
-      <c r="C39" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="D39" s="68" t="s">
-        <v>311</v>
-      </c>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="71" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="63" t="n">
+        <v>2600</v>
+      </c>
+      <c r="B39" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="E39" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F39" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G39" s="20"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C40" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D40" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="71" t="s">
+        <v>320</v>
+      </c>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="71"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="63" t="n">
+        <v>2800</v>
+      </c>
+      <c r="B41" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="E41" s="70" t="s">
+        <v>308</v>
+      </c>
+      <c r="F41" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="20"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C42" s="68" t="s">
         <v>315</v>
       </c>
-      <c r="H39" s="71"/>
-      <c r="I39" s="71"/>
-      <c r="J39" s="71"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="63" t="n">
-        <v>2600</v>
-      </c>
-      <c r="B40" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="D40" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="E40" s="66" t="s">
+      <c r="D42" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="71" t="s">
         <v>316</v>
       </c>
-      <c r="F40" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A41" s="11" t="s">
-        <v>317</v>
-      </c>
-      <c r="B41" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C41" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D41" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="71" t="s">
+      <c r="H42" s="71"/>
+      <c r="I42" s="71"/>
+      <c r="J42" s="71"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="63" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B43" s="64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D43" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="E43" s="70" t="s">
+        <v>308</v>
+      </c>
+      <c r="F43" s="67" t="s">
+        <v>232</v>
+      </c>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="20"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="B44" s="35" t="s">
         <v>319</v>
       </c>
-      <c r="H41" s="71"/>
-      <c r="I41" s="71"/>
-      <c r="J41" s="71"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="63" t="n">
-        <v>2800</v>
-      </c>
-      <c r="B42" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="D42" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="E42" s="70" t="s">
-        <v>307</v>
-      </c>
-      <c r="F42" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A43" s="11" t="s">
-        <v>320</v>
-      </c>
-      <c r="B43" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C43" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="D43" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="71" t="s">
+      <c r="C44" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D44" s="68" t="s">
         <v>315</v>
       </c>
-      <c r="H43" s="71"/>
-      <c r="I43" s="71"/>
-      <c r="J43" s="71"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="63" t="n">
-        <v>3000</v>
-      </c>
-      <c r="B44" s="64" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="D44" s="20" t="s">
-        <v>321</v>
-      </c>
-      <c r="E44" s="70" t="s">
-        <v>307</v>
-      </c>
-      <c r="F44" s="67" t="s">
-        <v>232</v>
-      </c>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="69"/>
+      <c r="H44" s="69"/>
+      <c r="I44" s="69"/>
+      <c r="J44" s="69"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B45" s="35" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C45" s="68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D45" s="68" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="E45" s="22"/>
       <c r="F45" s="22"/>
@@ -18977,16 +19146,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B46" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C46" s="68" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
       <c r="D46" s="68" t="s">
-        <v>324</v>
+        <v>305</v>
       </c>
       <c r="E46" s="22"/>
       <c r="F46" s="22"/>
@@ -18995,394 +19164,394 @@
       <c r="I46" s="69"/>
       <c r="J46" s="69"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A47" s="11" t="s">
-        <v>325</v>
-      </c>
-      <c r="B47" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C47" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="D47" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="69"/>
-      <c r="H47" s="69"/>
-      <c r="I47" s="69"/>
-      <c r="J47" s="69"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="25" t="s">
-        <v>326</v>
-      </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="28"/>
-      <c r="G49" s="28"/>
-      <c r="H49" s="28"/>
-      <c r="I49" s="28"/>
-      <c r="J49" s="28"/>
-    </row>
-    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
+      <c r="G48" s="28"/>
+      <c r="H48" s="28"/>
+      <c r="I48" s="28"/>
+      <c r="J48" s="28"/>
+    </row>
+    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B50" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C50" s="3" t="s">
+      <c r="B49" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="C49" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="D49" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F50" s="3" t="s">
+      <c r="E49" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3" t="s">
+      <c r="F49" s="3" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="63" t="n">
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="63" t="n">
         <v>1500</v>
       </c>
-      <c r="B51" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>327</v>
-      </c>
-      <c r="E51" s="66" t="s">
+      <c r="B50" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="F51" s="67" t="s">
+      <c r="D50" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="E50" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F50" s="67" t="s">
+        <v>302</v>
+      </c>
+      <c r="G50" s="20"/>
+      <c r="H50" s="20"/>
+      <c r="I50" s="20"/>
+      <c r="J50" s="20"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A51" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="B51" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C51" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D51" s="68" t="s">
+        <v>330</v>
+      </c>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="71" t="s">
+        <v>331</v>
+      </c>
+      <c r="H51" s="71"/>
+      <c r="I51" s="71"/>
+      <c r="J51" s="71"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="63" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B52" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A52" s="11" t="s">
+      <c r="D52" s="20" t="s">
         <v>328</v>
       </c>
-      <c r="B52" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C52" s="68" t="s">
+      <c r="E52" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F52" s="67" t="s">
+        <v>302</v>
+      </c>
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A53" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="B53" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C53" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D53" s="68" t="s">
+        <v>330</v>
+      </c>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="69"/>
+      <c r="H53" s="69"/>
+      <c r="I53" s="69"/>
+      <c r="J53" s="69"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="63" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B54" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="D52" s="68" t="s">
-        <v>329</v>
-      </c>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="71" t="s">
+      <c r="D54" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="E54" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F54" s="67" t="s">
+        <v>302</v>
+      </c>
+      <c r="G54" s="20"/>
+      <c r="H54" s="20"/>
+      <c r="I54" s="20"/>
+      <c r="J54" s="20"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A55" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="B55" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C55" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D55" s="68" t="s">
         <v>330</v>
       </c>
-      <c r="H52" s="71"/>
-      <c r="I52" s="71"/>
-      <c r="J52" s="71"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="63" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B53" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D53" s="20" t="s">
-        <v>327</v>
-      </c>
-      <c r="E53" s="66" t="s">
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="69"/>
+      <c r="H55" s="69"/>
+      <c r="I55" s="69"/>
+      <c r="J55" s="69"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="63" t="n">
+        <v>2800</v>
+      </c>
+      <c r="B56" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D56" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="E56" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F56" s="67" t="s">
+        <v>309</v>
+      </c>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A57" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="B57" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C57" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D57" s="68" t="s">
+        <v>312</v>
+      </c>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="71" t="s">
+        <v>335</v>
+      </c>
+      <c r="H57" s="71"/>
+      <c r="I57" s="71"/>
+      <c r="J57" s="71"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="63" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B58" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="F53" s="67" t="s">
-        <v>301</v>
-      </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A54" s="11" t="s">
-        <v>331</v>
-      </c>
-      <c r="B54" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C54" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D54" s="68" t="s">
-        <v>329</v>
-      </c>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="69"/>
-      <c r="H54" s="69"/>
-      <c r="I54" s="69"/>
-      <c r="J54" s="69"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="63" t="n">
-        <v>2500</v>
-      </c>
-      <c r="B55" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D55" s="20" t="s">
-        <v>327</v>
-      </c>
-      <c r="E55" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F55" s="67" t="s">
-        <v>301</v>
-      </c>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="20"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A56" s="11" t="s">
-        <v>332</v>
-      </c>
-      <c r="B56" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C56" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D56" s="68" t="s">
-        <v>329</v>
-      </c>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="69"/>
-      <c r="H56" s="69"/>
-      <c r="I56" s="69"/>
-      <c r="J56" s="69"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="63" t="n">
-        <v>2800</v>
-      </c>
-      <c r="B57" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" s="20" t="s">
+      <c r="D58" s="20" t="s">
+        <v>336</v>
+      </c>
+      <c r="E58" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F58" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="D57" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E57" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F57" s="67" t="s">
-        <v>308</v>
-      </c>
-      <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A58" s="11" t="s">
-        <v>333</v>
-      </c>
-      <c r="B58" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C58" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D58" s="68" t="s">
+      <c r="G58" s="20"/>
+      <c r="H58" s="20"/>
+      <c r="I58" s="20"/>
+      <c r="J58" s="20"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A59" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="B59" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="71" t="s">
-        <v>334</v>
-      </c>
-      <c r="H58" s="71"/>
-      <c r="I58" s="71"/>
-      <c r="J58" s="71"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="63" t="n">
-        <v>3000</v>
-      </c>
-      <c r="B59" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C59" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D59" s="20" t="s">
-        <v>335</v>
-      </c>
-      <c r="E59" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F59" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G59" s="20"/>
-      <c r="H59" s="20"/>
-      <c r="I59" s="20"/>
-      <c r="J59" s="20"/>
+      <c r="C59" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D59" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="71" t="s">
+        <v>338</v>
+      </c>
+      <c r="H59" s="71"/>
+      <c r="I59" s="71"/>
+      <c r="J59" s="71"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="B60" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C60" s="68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D60" s="68" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="E60" s="22"/>
       <c r="F60" s="22"/>
-      <c r="G60" s="71" t="s">
-        <v>337</v>
-      </c>
-      <c r="H60" s="71"/>
-      <c r="I60" s="71"/>
-      <c r="J60" s="71"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A61" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="B61" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C61" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D61" s="68" t="s">
+      <c r="G60" s="69"/>
+      <c r="H60" s="69"/>
+      <c r="I60" s="69"/>
+      <c r="J60" s="69"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="63" t="n">
+        <v>3100</v>
+      </c>
+      <c r="B61" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D61" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="E61" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F61" s="67" t="s">
+        <v>309</v>
+      </c>
+      <c r="G61" s="20"/>
+      <c r="H61" s="20"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A62" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="B62" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C62" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D62" s="68" t="s">
+        <v>312</v>
+      </c>
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="71" t="s">
+        <v>340</v>
+      </c>
+      <c r="H62" s="71"/>
+      <c r="I62" s="71"/>
+      <c r="J62" s="71"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="63" t="n">
+        <v>3500</v>
+      </c>
+      <c r="B63" s="64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" s="20" t="s">
+        <v>341</v>
+      </c>
+      <c r="D63" s="20" t="s">
+        <v>342</v>
+      </c>
+      <c r="E63" s="70" t="s">
+        <v>308</v>
+      </c>
+      <c r="F63" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G63" s="20"/>
+      <c r="H63" s="20"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A64" s="11" t="s">
+        <v>343</v>
+      </c>
+      <c r="B64" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="69"/>
-      <c r="H61" s="69"/>
-      <c r="I61" s="69"/>
-      <c r="J61" s="69"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="63" t="n">
-        <v>3100</v>
-      </c>
-      <c r="B62" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="D62" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E62" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F62" s="67" t="s">
-        <v>308</v>
-      </c>
-      <c r="G62" s="20"/>
-      <c r="H62" s="20"/>
-      <c r="I62" s="20"/>
-      <c r="J62" s="20"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A63" s="11" t="s">
-        <v>338</v>
-      </c>
-      <c r="B63" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C63" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D63" s="68" t="s">
-        <v>311</v>
-      </c>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="71" t="s">
-        <v>339</v>
-      </c>
-      <c r="H63" s="71"/>
-      <c r="I63" s="71"/>
-      <c r="J63" s="71"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="63" t="n">
-        <v>3500</v>
-      </c>
-      <c r="B64" s="64" t="n">
-        <v>4</v>
-      </c>
-      <c r="C64" s="20" t="s">
-        <v>340</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>341</v>
-      </c>
-      <c r="E64" s="70" t="s">
-        <v>307</v>
-      </c>
-      <c r="F64" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
+      <c r="C64" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D64" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="69"/>
+      <c r="H64" s="69"/>
+      <c r="I64" s="69"/>
+      <c r="J64" s="69"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B65" s="35" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="C65" s="68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D65" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E65" s="22"/>
       <c r="F65" s="22"/>
@@ -19393,192 +19562,192 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>344</v>
+        <v>311</v>
       </c>
       <c r="C66" s="68" t="s">
-        <v>301</v>
+        <v>325</v>
       </c>
       <c r="D66" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E66" s="22"/>
       <c r="F66" s="22"/>
-      <c r="G66" s="69"/>
-      <c r="H66" s="69"/>
-      <c r="I66" s="69"/>
-      <c r="J66" s="69"/>
+      <c r="G66" s="71" t="s">
+        <v>340</v>
+      </c>
+      <c r="H66" s="71"/>
+      <c r="I66" s="71"/>
+      <c r="J66" s="71"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>345</v>
+        <v>314</v>
       </c>
       <c r="B67" s="35" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C67" s="68" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="D67" s="68" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="E67" s="22"/>
       <c r="F67" s="22"/>
       <c r="G67" s="71" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="H67" s="71"/>
       <c r="I67" s="71"/>
       <c r="J67" s="71"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A68" s="11" t="s">
-        <v>313</v>
-      </c>
-      <c r="B68" s="35" t="s">
-        <v>303</v>
-      </c>
-      <c r="C68" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="D68" s="68" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="63" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B68" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D68" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="E68" s="70" t="s">
+        <v>308</v>
+      </c>
+      <c r="F68" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G68" s="20"/>
+      <c r="H68" s="20"/>
+      <c r="I68" s="20"/>
+      <c r="J68" s="20"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A69" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="B69" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="E68" s="22"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="71" t="s">
-        <v>346</v>
-      </c>
-      <c r="H68" s="71"/>
-      <c r="I68" s="71"/>
-      <c r="J68" s="71"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="63" t="n">
-        <v>4000</v>
-      </c>
-      <c r="B69" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C69" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="D69" s="20" t="s">
+      <c r="C69" s="68" t="s">
+        <v>315</v>
+      </c>
+      <c r="D69" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E69" s="22"/>
+      <c r="F69" s="22"/>
+      <c r="G69" s="69"/>
+      <c r="H69" s="69"/>
+      <c r="I69" s="69"/>
+      <c r="J69" s="69"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="63" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B70" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="65" t="s">
+        <v>301</v>
+      </c>
+      <c r="D70" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E69" s="70" t="s">
-        <v>307</v>
-      </c>
-      <c r="F69" s="67" t="s">
+      <c r="E70" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F70" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G69" s="20"/>
-      <c r="H69" s="20"/>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A70" s="11" t="s">
-        <v>325</v>
-      </c>
-      <c r="B70" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C70" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="D70" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="69"/>
-      <c r="H70" s="69"/>
-      <c r="I70" s="69"/>
-      <c r="J70" s="69"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="63" t="n">
-        <v>5000</v>
-      </c>
-      <c r="B71" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C71" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D71" s="20" t="s">
+      <c r="G70" s="20"/>
+      <c r="H70" s="20"/>
+      <c r="I70" s="20"/>
+      <c r="J70" s="20"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A71" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="B71" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C71" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D71" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E71" s="22"/>
+      <c r="F71" s="22"/>
+      <c r="G71" s="69"/>
+      <c r="H71" s="69"/>
+      <c r="I71" s="69"/>
+      <c r="J71" s="69"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="63" t="n">
+        <v>5500</v>
+      </c>
+      <c r="B72" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" s="65" t="s">
+        <v>301</v>
+      </c>
+      <c r="D72" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="E72" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F72" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="E71" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F71" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G71" s="20"/>
-      <c r="H71" s="20"/>
-      <c r="I71" s="20"/>
-      <c r="J71" s="20"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A72" s="11" t="s">
-        <v>322</v>
-      </c>
-      <c r="B72" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C72" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D72" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E72" s="22"/>
-      <c r="F72" s="22"/>
-      <c r="G72" s="69"/>
-      <c r="H72" s="69"/>
-      <c r="I72" s="69"/>
-      <c r="J72" s="69"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="63" t="n">
-        <v>5500</v>
-      </c>
-      <c r="B73" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D73" s="20" t="s">
-        <v>347</v>
-      </c>
-      <c r="E73" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F73" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G73" s="20"/>
-      <c r="H73" s="20"/>
-      <c r="I73" s="20"/>
-      <c r="J73" s="20"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="20"/>
+      <c r="I72" s="20"/>
+      <c r="J72" s="20"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A73" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="B73" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C73" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D73" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E73" s="22"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="69"/>
+      <c r="H73" s="69"/>
+      <c r="I73" s="69"/>
+      <c r="J73" s="69"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A74" s="11" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B74" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C74" s="68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D74" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E74" s="22"/>
       <c r="F74" s="22"/>
@@ -19587,146 +19756,146 @@
       <c r="I74" s="69"/>
       <c r="J74" s="69"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A75" s="11" t="s">
-        <v>349</v>
-      </c>
-      <c r="B75" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C75" s="68" t="s">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="63" t="n">
+        <v>6000</v>
+      </c>
+      <c r="B75" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="D75" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="69"/>
-      <c r="H75" s="69"/>
-      <c r="I75" s="69"/>
-      <c r="J75" s="69"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="63" t="n">
-        <v>6000</v>
-      </c>
-      <c r="B76" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C76" s="65" t="s">
+      <c r="D75" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="E75" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F75" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G75" s="20"/>
+      <c r="H75" s="20"/>
+      <c r="I75" s="20"/>
+      <c r="J75" s="20"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A76" s="11" t="s">
+        <v>351</v>
+      </c>
+      <c r="B76" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C76" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D76" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E76" s="22"/>
+      <c r="F76" s="22"/>
+      <c r="G76" s="69"/>
+      <c r="H76" s="69"/>
+      <c r="I76" s="69"/>
+      <c r="J76" s="69"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="25" t="s">
+        <v>352</v>
+      </c>
+      <c r="B78" s="28"/>
+      <c r="C78" s="28"/>
+      <c r="D78" s="28"/>
+      <c r="E78" s="28"/>
+      <c r="F78" s="28"/>
+      <c r="G78" s="28"/>
+      <c r="H78" s="28"/>
+      <c r="I78" s="28"/>
+      <c r="J78" s="28"/>
+    </row>
+    <row r="79" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="D76" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="E76" s="66" t="s">
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="63" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B80" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="F76" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G76" s="20"/>
-      <c r="H76" s="20"/>
-      <c r="I76" s="20"/>
-      <c r="J76" s="20"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A77" s="11" t="s">
-        <v>350</v>
-      </c>
-      <c r="B77" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C77" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D77" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="69"/>
-      <c r="H77" s="69"/>
-      <c r="I77" s="69"/>
-      <c r="J77" s="69"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="25" t="s">
-        <v>351</v>
-      </c>
-      <c r="B79" s="28"/>
-      <c r="C79" s="28"/>
-      <c r="D79" s="28"/>
-      <c r="E79" s="28"/>
-      <c r="F79" s="28"/>
-      <c r="G79" s="28"/>
-      <c r="H79" s="28"/>
-      <c r="I79" s="28"/>
-      <c r="J79" s="28"/>
-    </row>
-    <row r="80" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="E80" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="G80" s="3"/>
-      <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
-      <c r="J80" s="3" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="63" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B81" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C81" s="65" t="s">
-        <v>300</v>
-      </c>
-      <c r="D81" s="20" t="s">
-        <v>352</v>
-      </c>
-      <c r="E81" s="66" t="s">
-        <v>301</v>
-      </c>
-      <c r="F81" s="67" t="s">
-        <v>301</v>
-      </c>
-      <c r="G81" s="20"/>
-      <c r="H81" s="20"/>
-      <c r="I81" s="20"/>
-      <c r="J81" s="20"/>
+      <c r="D80" s="20" t="s">
+        <v>353</v>
+      </c>
+      <c r="E80" s="66" t="s">
+        <v>302</v>
+      </c>
+      <c r="F80" s="67" t="s">
+        <v>302</v>
+      </c>
+      <c r="G80" s="20"/>
+      <c r="H80" s="20"/>
+      <c r="I80" s="20"/>
+      <c r="J80" s="20"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A81" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="B81" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C81" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="D81" s="68" t="s">
+        <v>330</v>
+      </c>
+      <c r="E81" s="22"/>
+      <c r="F81" s="22"/>
+      <c r="G81" s="69"/>
+      <c r="H81" s="69"/>
+      <c r="I81" s="69"/>
+      <c r="J81" s="69"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A82" s="11" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B82" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C82" s="68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D82" s="68" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E82" s="22"/>
       <c r="F82" s="22"/>
@@ -19735,362 +19904,342 @@
       <c r="I82" s="69"/>
       <c r="J82" s="69"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A83" s="11" t="s">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="63" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B83" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D83" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="E83" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F83" s="67" t="s">
+        <v>232</v>
+      </c>
+      <c r="G83" s="20"/>
+      <c r="H83" s="20"/>
+      <c r="I83" s="20"/>
+      <c r="J83" s="20"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A84" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="B84" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C84" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D84" s="68" t="s">
+        <v>315</v>
+      </c>
+      <c r="E84" s="22"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="69"/>
+      <c r="H84" s="69"/>
+      <c r="I84" s="69"/>
+      <c r="J84" s="69"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="63" t="n">
+        <v>2800</v>
+      </c>
+      <c r="B85" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D85" s="20" t="s">
+        <v>355</v>
+      </c>
+      <c r="E85" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F85" s="67" t="s">
+        <v>355</v>
+      </c>
+      <c r="G85" s="20"/>
+      <c r="H85" s="20"/>
+      <c r="I85" s="20"/>
+      <c r="J85" s="20"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A86" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="B86" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C86" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D86" s="68" t="s">
+        <v>357</v>
+      </c>
+      <c r="E86" s="22"/>
+      <c r="F86" s="22"/>
+      <c r="G86" s="71" t="s">
+        <v>358</v>
+      </c>
+      <c r="H86" s="71"/>
+      <c r="I86" s="71"/>
+      <c r="J86" s="71"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="63" t="n">
+        <v>3100</v>
+      </c>
+      <c r="B87" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" s="20" t="s">
+        <v>359</v>
+      </c>
+      <c r="D87" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="E87" s="66" t="s">
+        <v>360</v>
+      </c>
+      <c r="F87" s="67" t="s">
+        <v>309</v>
+      </c>
+      <c r="G87" s="20"/>
+      <c r="H87" s="20"/>
+      <c r="I87" s="20"/>
+      <c r="J87" s="20"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A88" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="B88" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="C88" s="68" t="s">
         <v>325</v>
       </c>
-      <c r="B83" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C83" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="D83" s="68" t="s">
-        <v>329</v>
-      </c>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="69"/>
-      <c r="H83" s="69"/>
-      <c r="I83" s="69"/>
-      <c r="J83" s="69"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="63" t="n">
-        <v>2500</v>
-      </c>
-      <c r="B84" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C84" s="20" t="s">
+      <c r="D88" s="68" t="s">
+        <v>312</v>
+      </c>
+      <c r="E88" s="22"/>
+      <c r="F88" s="22"/>
+      <c r="G88" s="71" t="s">
+        <v>362</v>
+      </c>
+      <c r="H88" s="71"/>
+      <c r="I88" s="71"/>
+      <c r="J88" s="71"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="63" t="n">
+        <v>3500</v>
+      </c>
+      <c r="B89" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="D89" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="E89" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F89" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="D84" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="E84" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F84" s="67" t="s">
-        <v>232</v>
-      </c>
-      <c r="G84" s="20"/>
-      <c r="H84" s="20"/>
-      <c r="I84" s="20"/>
-      <c r="J84" s="20"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A85" s="11" t="s">
-        <v>353</v>
-      </c>
-      <c r="B85" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C85" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D85" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
-      <c r="G85" s="69"/>
-      <c r="H85" s="69"/>
-      <c r="I85" s="69"/>
-      <c r="J85" s="69"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="63" t="n">
-        <v>2800</v>
-      </c>
-      <c r="B86" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C86" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="D86" s="20" t="s">
-        <v>354</v>
-      </c>
-      <c r="E86" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F86" s="67" t="s">
-        <v>354</v>
-      </c>
-      <c r="G86" s="20"/>
-      <c r="H86" s="20"/>
-      <c r="I86" s="20"/>
-      <c r="J86" s="20"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A87" s="11" t="s">
-        <v>355</v>
-      </c>
-      <c r="B87" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C87" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D87" s="68" t="s">
-        <v>356</v>
-      </c>
-      <c r="E87" s="22"/>
-      <c r="F87" s="22"/>
-      <c r="G87" s="71" t="s">
-        <v>357</v>
-      </c>
-      <c r="H87" s="71"/>
-      <c r="I87" s="71"/>
-      <c r="J87" s="71"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="63" t="n">
-        <v>3100</v>
-      </c>
-      <c r="B88" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C88" s="20" t="s">
-        <v>358</v>
-      </c>
-      <c r="D88" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E88" s="66" t="s">
-        <v>359</v>
-      </c>
-      <c r="F88" s="67" t="s">
-        <v>308</v>
-      </c>
-      <c r="G88" s="20"/>
-      <c r="H88" s="20"/>
-      <c r="I88" s="20"/>
-      <c r="J88" s="20"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A89" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="B89" s="35" t="s">
-        <v>318</v>
-      </c>
-      <c r="C89" s="68" t="s">
-        <v>324</v>
-      </c>
-      <c r="D89" s="68" t="s">
+      <c r="G89" s="20"/>
+      <c r="H89" s="20"/>
+      <c r="I89" s="20"/>
+      <c r="J89" s="20"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A90" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="B90" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="E89" s="22"/>
-      <c r="F89" s="22"/>
-      <c r="G89" s="71" t="s">
-        <v>361</v>
-      </c>
-      <c r="H89" s="71"/>
-      <c r="I89" s="71"/>
-      <c r="J89" s="71"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="63" t="n">
-        <v>3500</v>
-      </c>
-      <c r="B90" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C90" s="20" t="s">
-        <v>347</v>
-      </c>
-      <c r="D90" s="20" t="s">
-        <v>347</v>
-      </c>
-      <c r="E90" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F90" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G90" s="20"/>
-      <c r="H90" s="20"/>
-      <c r="I90" s="20"/>
-      <c r="J90" s="20"/>
+      <c r="C90" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D90" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E90" s="22"/>
+      <c r="F90" s="22"/>
+      <c r="G90" s="71" t="s">
+        <v>363</v>
+      </c>
+      <c r="H90" s="71"/>
+      <c r="I90" s="71"/>
+      <c r="J90" s="71"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>345</v>
+        <v>314</v>
       </c>
       <c r="B91" s="35" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C91" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D91" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E91" s="22"/>
       <c r="F91" s="22"/>
       <c r="G91" s="71" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="H91" s="71"/>
       <c r="I91" s="71"/>
       <c r="J91" s="71"/>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A92" s="11" t="s">
-        <v>313</v>
-      </c>
-      <c r="B92" s="35" t="s">
-        <v>303</v>
-      </c>
-      <c r="C92" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D92" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E92" s="22"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="71" t="s">
-        <v>363</v>
-      </c>
-      <c r="H92" s="71"/>
-      <c r="I92" s="71"/>
-      <c r="J92" s="71"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="63" t="n">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="63" t="n">
         <v>3700</v>
       </c>
-      <c r="B93" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C93" s="20" t="s">
-        <v>358</v>
-      </c>
-      <c r="D93" s="20" t="s">
+      <c r="B92" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" s="20" t="s">
+        <v>359</v>
+      </c>
+      <c r="D92" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E93" s="66" t="s">
-        <v>359</v>
-      </c>
-      <c r="F93" s="67" t="s">
+      <c r="E92" s="66" t="s">
+        <v>360</v>
+      </c>
+      <c r="F92" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="G93" s="20"/>
-      <c r="H93" s="20"/>
-      <c r="I93" s="20"/>
-      <c r="J93" s="20"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A94" s="11" t="s">
+      <c r="G92" s="20"/>
+      <c r="H92" s="20"/>
+      <c r="I92" s="20"/>
+      <c r="J92" s="20"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A93" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="B93" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C93" s="68" t="s">
+        <v>325</v>
+      </c>
+      <c r="D93" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E93" s="22"/>
+      <c r="F93" s="22"/>
+      <c r="G93" s="71" t="s">
+        <v>362</v>
+      </c>
+      <c r="H93" s="71"/>
+      <c r="I93" s="71"/>
+      <c r="J93" s="71"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="63" t="n">
+        <v>3900</v>
+      </c>
+      <c r="B94" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D94" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="E94" s="66" t="s">
+        <v>317</v>
+      </c>
+      <c r="F94" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G94" s="20"/>
+      <c r="H94" s="20"/>
+      <c r="I94" s="20"/>
+      <c r="J94" s="20"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A95" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B95" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="C95" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="D95" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="E95" s="22"/>
+      <c r="F95" s="22"/>
+      <c r="G95" s="71" t="s">
         <v>364</v>
       </c>
-      <c r="B94" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C94" s="68" t="s">
-        <v>324</v>
-      </c>
-      <c r="D94" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E94" s="22"/>
-      <c r="F94" s="22"/>
-      <c r="G94" s="71" t="s">
-        <v>361</v>
-      </c>
-      <c r="H94" s="71"/>
-      <c r="I94" s="71"/>
-      <c r="J94" s="71"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="63" t="n">
-        <v>3900</v>
-      </c>
-      <c r="B95" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C95" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="D95" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="E95" s="66" t="s">
-        <v>316</v>
-      </c>
-      <c r="F95" s="67" t="s">
-        <v>239</v>
-      </c>
-      <c r="G95" s="20"/>
-      <c r="H95" s="20"/>
-      <c r="I95" s="20"/>
-      <c r="J95" s="20"/>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A96" s="11" t="s">
-        <v>365</v>
-      </c>
-      <c r="B96" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="C96" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="D96" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="E96" s="22"/>
-      <c r="F96" s="22"/>
-      <c r="G96" s="71" t="s">
-        <v>363</v>
-      </c>
-      <c r="H96" s="71"/>
-      <c r="I96" s="71"/>
-      <c r="J96" s="71"/>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="s">
-        <v>366</v>
+      <c r="H95" s="71"/>
+      <c r="I95" s="71"/>
+      <c r="J95" s="71"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="G37:J37"/>
     <mergeCell ref="G38:J38"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="G41:J41"/>
-    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="G44:J44"/>
     <mergeCell ref="G45:J45"/>
     <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G52:J52"/>
-    <mergeCell ref="G54:J54"/>
-    <mergeCell ref="G56:J56"/>
-    <mergeCell ref="G58:J58"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G55:J55"/>
+    <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G59:J59"/>
     <mergeCell ref="G60:J60"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="G63:J63"/>
+    <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G64:J64"/>
     <mergeCell ref="G65:J65"/>
     <mergeCell ref="G66:J66"/>
     <mergeCell ref="G67:J67"/>
-    <mergeCell ref="G68:J68"/>
-    <mergeCell ref="G70:J70"/>
-    <mergeCell ref="G72:J72"/>
+    <mergeCell ref="G69:J69"/>
+    <mergeCell ref="G71:J71"/>
+    <mergeCell ref="G73:J73"/>
     <mergeCell ref="G74:J74"/>
-    <mergeCell ref="G75:J75"/>
-    <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G81:J81"/>
     <mergeCell ref="G82:J82"/>
-    <mergeCell ref="G83:J83"/>
-    <mergeCell ref="G85:J85"/>
-    <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G89:J89"/>
+    <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G86:J86"/>
+    <mergeCell ref="G88:J88"/>
+    <mergeCell ref="G90:J90"/>
     <mergeCell ref="G91:J91"/>
-    <mergeCell ref="G92:J92"/>
-    <mergeCell ref="G94:J94"/>
-    <mergeCell ref="G96:J96"/>
+    <mergeCell ref="G93:J93"/>
+    <mergeCell ref="G95:J95"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>